<commit_message>
adding drop down, changing modelingg excel, and updating main
Former-commit-id: 79ff115eaaaa98f355490297351c676acad41994
</commit_message>
<xml_diff>
--- a/images/wsp/Financial-Model.xlsx
+++ b/images/wsp/Financial-Model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conno\OneDrive\Desktop\Wall Street Prep\Financial-Statement-Modeling-DL-Kit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Website\connorbuttonweb.github.io\images\wsp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C09AA7-9256-49C9-98E0-B06477C26871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD818F9F-D227-4721-A30E-EE783B25433A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" tabRatio="736" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" firstSheet="16" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FSM Data Input_Empty" sheetId="66" r:id="rId1"/>
@@ -32,7 +32,6 @@
     <sheet name="FSM + Schedules" sheetId="78" r:id="rId17"/>
     <sheet name="FSM 2019 Update Empty" sheetId="86" r:id="rId18"/>
     <sheet name="2019 FSM Update Complete" sheetId="84" r:id="rId19"/>
-    <sheet name="Sheet1" sheetId="87" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="CIQWBGuid" hidden="1">"a611639b-bab1-425e-aaa5-008c326fdfdb"</definedName>
@@ -3227,7 +3226,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3467" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3455" uniqueCount="338">
   <si>
     <t>Tax rate</t>
   </si>
@@ -4301,33 +4300,6 @@
   </si>
   <si>
     <t>Commercial paper / revolver*</t>
-  </si>
-  <si>
-    <t>Share Based Compensation</t>
-  </si>
-  <si>
-    <t>Answer</t>
-  </si>
-  <si>
-    <t>Ammortization expense</t>
-  </si>
-  <si>
-    <t>SG&amp;A</t>
-  </si>
-  <si>
-    <t>EBIT</t>
-  </si>
-  <si>
-    <t>EBIT margin</t>
-  </si>
-  <si>
-    <t>Revenu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accounts Receivable </t>
-  </si>
-  <si>
-    <t>%</t>
   </si>
 </sst>
 </file>
@@ -6167,7 +6139,7 @@
     <xf numFmtId="0" fontId="82" fillId="0" borderId="0" applyAlignment="0"/>
     <xf numFmtId="238" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="293">
+  <cellXfs count="291">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="62" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6589,8 +6561,6 @@
     <xf numFmtId="246" fontId="60" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="229" fontId="65" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="246" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="246" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="199" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="209">
     <cellStyle name="$" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -7648,23 +7618,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O112"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.26953125" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" customWidth="1"/>
+    <col min="9" max="9" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1"/>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1">
+    <row r="1" spans="1:12" ht="15" thickBot="1"/>
+    <row r="2" spans="1:12" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -8738,21 +8708,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:T219"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="11" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="11" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -12787,7 +12757,7 @@
     <row r="160" spans="3:18">
       <c r="C160" s="16"/>
     </row>
-    <row r="161" spans="3:16" ht="15.75" thickBot="1">
+    <row r="161" spans="3:16" ht="15" thickBot="1">
       <c r="C161" s="44" t="s">
         <v>188</v>
       </c>
@@ -12931,8 +12901,8 @@
       <c r="J171" s="5"/>
       <c r="K171" s="5"/>
     </row>
-    <row r="172" spans="3:16" ht="15.75" thickBot="1"/>
-    <row r="173" spans="3:16" ht="15.75" thickBot="1">
+    <row r="172" spans="3:16" ht="15" thickBot="1"/>
+    <row r="173" spans="3:16" ht="15" thickBot="1">
       <c r="C173" t="s">
         <v>193</v>
       </c>
@@ -13483,7 +13453,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="195" spans="3:13" ht="15.75" thickBot="1">
+    <row r="195" spans="3:13" ht="15" thickBot="1">
       <c r="C195" s="49" t="s">
         <v>85</v>
       </c>
@@ -14162,21 +14132,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:T222"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="1:19" ht="15.75" thickBot="1">
+    <row r="1" spans="1:19" ht="15" thickBot="1"/>
+    <row r="2" spans="1:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -18289,7 +18259,7 @@
     <row r="160" spans="3:18">
       <c r="C160" s="16"/>
     </row>
-    <row r="161" spans="3:16" ht="15.75" thickBot="1">
+    <row r="161" spans="3:16" ht="15" thickBot="1">
       <c r="C161" s="44" t="s">
         <v>188</v>
       </c>
@@ -18475,8 +18445,8 @@
       <c r="J171" s="5"/>
       <c r="K171" s="5"/>
     </row>
-    <row r="172" spans="3:16" ht="15.75" thickBot="1"/>
-    <row r="173" spans="3:16" ht="15.75" thickBot="1">
+    <row r="172" spans="3:16" ht="15" thickBot="1"/>
+    <row r="173" spans="3:16" ht="15" thickBot="1">
       <c r="C173" t="s">
         <v>193</v>
       </c>
@@ -19031,7 +19001,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="195" spans="3:13" ht="15.75" thickBot="1">
+    <row r="195" spans="3:13" ht="15" thickBot="1">
       <c r="C195" s="49" t="s">
         <v>85</v>
       </c>
@@ -19461,7 +19431,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="212" spans="3:13" ht="15.75" thickBot="1">
+    <row r="212" spans="3:13" ht="15" thickBot="1">
       <c r="C212" s="281" t="s">
         <v>327</v>
       </c>
@@ -19594,7 +19564,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="217" spans="3:13" ht="15.75" thickBot="1">
+    <row r="217" spans="3:13" ht="15" thickBot="1">
       <c r="C217" s="281" t="s">
         <v>328</v>
       </c>
@@ -19726,14 +19696,14 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C2:R54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="2.5703125" customWidth="1"/>
-    <col min="14" max="14" width="29.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="11" width="10.81640625" customWidth="1"/>
+    <col min="12" max="12" width="2.54296875" customWidth="1"/>
+    <col min="14" max="14" width="29.54296875" bestFit="1" customWidth="1"/>
     <col min="15" max="19" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -20845,15 +20815,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C2:R54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="2.5703125" customWidth="1"/>
-    <col min="14" max="14" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="11" width="10.81640625" customWidth="1"/>
+    <col min="12" max="12" width="2.54296875" customWidth="1"/>
+    <col min="14" max="14" width="29.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -21944,15 +21914,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C2:P54"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="2.5703125" customWidth="1"/>
-    <col min="14" max="14" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="11" width="10.81640625" customWidth="1"/>
+    <col min="12" max="12" width="2.54296875" customWidth="1"/>
+    <col min="14" max="14" width="29.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -23042,21 +23012,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:T216"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="58.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:19" ht="15.75" thickBot="1">
+    <row r="1" spans="2:19" ht="15" thickBot="1"/>
+    <row r="2" spans="2:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -27122,7 +27092,7 @@
     <row r="160" spans="3:18">
       <c r="C160" s="16"/>
     </row>
-    <row r="161" spans="2:16" ht="15.75" thickBot="1">
+    <row r="161" spans="2:16" ht="15" thickBot="1">
       <c r="C161" s="44" t="s">
         <v>188</v>
       </c>
@@ -27311,8 +27281,8 @@
       <c r="J171" s="5"/>
       <c r="K171" s="5"/>
     </row>
-    <row r="172" spans="2:16" ht="15.75" thickBot="1"/>
-    <row r="173" spans="2:16" ht="15.75" thickBot="1">
+    <row r="172" spans="2:16" ht="15" thickBot="1"/>
+    <row r="173" spans="2:16" ht="15" thickBot="1">
       <c r="C173" t="s">
         <v>193</v>
       </c>
@@ -28036,7 +28006,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="200" spans="3:13" ht="15.75" thickBot="1">
+    <row r="200" spans="3:13" ht="15" thickBot="1">
       <c r="C200" s="49" t="s">
         <v>85</v>
       </c>
@@ -28505,23 +28475,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:AI282"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="2.28515625" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
-    <col min="16" max="16" width="11.85546875" customWidth="1"/>
-    <col min="17" max="19" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="58.26953125" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="2.26953125" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" customWidth="1"/>
+    <col min="16" max="16" width="11.81640625" customWidth="1"/>
+    <col min="17" max="19" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:35" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:35" ht="15.75" thickBot="1">
+    <row r="1" spans="3:35" ht="15" thickBot="1"/>
+    <row r="2" spans="3:35" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -29260,7 +29230,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="3:16" ht="14.45" customHeight="1">
+    <row r="32" spans="3:16" ht="14.5" customHeight="1">
       <c r="C32" s="27" t="s">
         <v>47</v>
       </c>
@@ -34177,7 +34147,7 @@
     <row r="226" spans="3:13">
       <c r="C226" s="16"/>
     </row>
-    <row r="227" spans="3:13" ht="15.75" thickBot="1">
+    <row r="227" spans="3:13" ht="15" thickBot="1">
       <c r="C227" s="44" t="s">
         <v>188</v>
       </c>
@@ -34364,8 +34334,8 @@
       <c r="K237" s="5"/>
       <c r="M237" s="16"/>
     </row>
-    <row r="238" spans="3:13" ht="15.75" thickBot="1"/>
-    <row r="239" spans="3:13" ht="15.75" thickBot="1">
+    <row r="238" spans="3:13" ht="15" thickBot="1"/>
+    <row r="239" spans="3:13" ht="15" thickBot="1">
       <c r="C239" t="s">
         <v>193</v>
       </c>
@@ -35086,7 +35056,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="266" spans="3:15" ht="15.75" thickBot="1">
+    <row r="266" spans="3:15" ht="15" thickBot="1">
       <c r="C266" s="49" t="s">
         <v>85</v>
       </c>
@@ -35575,23 +35545,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:V287"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="2.28515625" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
-    <col min="16" max="16" width="11.85546875" customWidth="1"/>
-    <col min="17" max="19" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="58.26953125" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="2.26953125" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" customWidth="1"/>
+    <col min="16" max="16" width="11.81640625" customWidth="1"/>
+    <col min="17" max="19" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:21" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:21" ht="15.75" thickBot="1">
+    <row r="1" spans="3:21" ht="15" thickBot="1"/>
+    <row r="2" spans="3:21" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -38376,7 +38346,7 @@
       <c r="L101" s="18"/>
       <c r="M101" s="18"/>
     </row>
-    <row r="102" spans="3:13" ht="14.45" customHeight="1">
+    <row r="102" spans="3:13" ht="14.5" customHeight="1">
       <c r="G102" s="140"/>
     </row>
     <row r="103" spans="3:13">
@@ -38868,7 +38838,7 @@
         <v>121.03085552459689</v>
       </c>
     </row>
-    <row r="127" spans="3:15" ht="14.45" customHeight="1">
+    <row r="127" spans="3:15" ht="14.5" customHeight="1">
       <c r="C127" s="16" t="s">
         <v>290</v>
       </c>
@@ -38897,7 +38867,7 @@
         <v>-44.804043820726136</v>
       </c>
     </row>
-    <row r="128" spans="3:15" ht="14.45" customHeight="1">
+    <row r="128" spans="3:15" ht="14.5" customHeight="1">
       <c r="C128" s="16"/>
       <c r="F128" s="211"/>
       <c r="G128" s="211"/>
@@ -41306,7 +41276,7 @@
     <row r="226" spans="3:13">
       <c r="C226" s="16"/>
     </row>
-    <row r="227" spans="3:13" ht="15.75" thickBot="1">
+    <row r="227" spans="3:13" ht="15" thickBot="1">
       <c r="C227" s="44" t="s">
         <v>188</v>
       </c>
@@ -41493,8 +41463,8 @@
       <c r="K237" s="5"/>
       <c r="M237" s="16"/>
     </row>
-    <row r="238" spans="3:13" ht="15.75" thickBot="1"/>
-    <row r="239" spans="3:13" ht="15.75" thickBot="1">
+    <row r="238" spans="3:13" ht="15" thickBot="1"/>
+    <row r="239" spans="3:13" ht="15" thickBot="1">
       <c r="C239" t="s">
         <v>193</v>
       </c>
@@ -42215,7 +42185,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="266" spans="3:15" ht="15.75" thickBot="1">
+    <row r="266" spans="3:15" ht="15" thickBot="1">
       <c r="C266" s="49" t="s">
         <v>85</v>
       </c>
@@ -42712,20 +42682,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:U180"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.7109375" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="1.7265625" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:20" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:20" ht="15.75" thickBot="1">
+    <row r="1" spans="3:20" ht="15" thickBot="1"/>
+    <row r="2" spans="3:20" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -47610,20 +47580,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:U203"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="12" width="11.42578125" customWidth="1"/>
-    <col min="13" max="13" width="3.28515625" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="12" width="11.453125" customWidth="1"/>
+    <col min="13" max="13" width="3.26953125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:20" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:20" ht="15.75" thickBot="1">
+    <row r="1" spans="3:20" ht="15" thickBot="1"/>
+    <row r="2" spans="3:20" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -52507,8 +52477,8 @@
       <c r="K179" s="5"/>
       <c r="L179" s="5"/>
     </row>
-    <row r="180" spans="3:14" ht="15.75" thickBot="1"/>
-    <row r="181" spans="3:14" ht="15.75" thickBot="1">
+    <row r="180" spans="3:14" ht="15" thickBot="1"/>
+    <row r="181" spans="3:14" ht="15" thickBot="1">
       <c r="C181" t="s">
         <v>193</v>
       </c>
@@ -53014,7 +52984,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="203" spans="3:12" ht="15.75" thickBot="1">
+    <row r="203" spans="3:12" ht="15" thickBot="1">
       <c r="C203" s="49" t="s">
         <v>85</v>
       </c>
@@ -53081,21 +53051,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:O75"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="2.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="7" width="2.26953125" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" customWidth="1"/>
+    <col min="10" max="12" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:8" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:8" ht="15.75" thickBot="1">
+    <row r="1" spans="3:8" ht="15" thickBot="1"/>
+    <row r="2" spans="3:8" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -54094,161 +54064,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEF37D56-3ED9-4E7B-9B0B-7E8A80022A19}">
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="9.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>338</v>
-      </c>
-      <c r="C1" s="291">
-        <v>34977</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="291">
-        <v>1302734</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>339</v>
-      </c>
-      <c r="C3" s="291">
-        <f>C2+C1</f>
-        <v>1337711</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>340</v>
-      </c>
-      <c r="C5">
-        <f>3603+3595+3584+3584+2911</f>
-        <v>17277</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="C7">
-        <f>ROUND((28519-1650)/5797,0)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>344</v>
-      </c>
-      <c r="C8">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9">
-        <f>10000*0.65</f>
-        <v>6500</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>341</v>
-      </c>
-      <c r="C10">
-        <f>-2000</f>
-        <v>-2000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>342</v>
-      </c>
-      <c r="C11">
-        <f>SUM(C9:C10)</f>
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>343</v>
-      </c>
-      <c r="C12">
-        <f>C11/C8</f>
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="C15" s="16">
-        <v>2013</v>
-      </c>
-      <c r="D15" s="16">
-        <v>2014</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="291">
-        <v>5000</v>
-      </c>
-      <c r="E16" s="291"/>
-      <c r="F16" s="291"/>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="16" t="s">
-        <v>345</v>
-      </c>
-      <c r="C17">
-        <v>400</v>
-      </c>
-      <c r="D17">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>346</v>
-      </c>
-      <c r="C19" s="292">
-        <f>AVERAGE(C17:D17)/D16</f>
-        <v>0.1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9BCE93C-4E65-4935-A6A4-F25878B0273E}">
   <dimension ref="C1:T120"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" customWidth="1"/>
+    <col min="5" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -57305,20 +57138,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:T92"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="1:19" ht="15.75" thickBot="1">
+    <row r="1" spans="1:19" ht="15" thickBot="1"/>
+    <row r="2" spans="1:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -59508,20 +59341,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{727A1621-455D-4421-A091-A6301FBCF730}">
   <dimension ref="C1:T122"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="11" width="12.7109375" customWidth="1"/>
-    <col min="12" max="12" width="2.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" customWidth="1"/>
+    <col min="4" max="11" width="12.7265625" customWidth="1"/>
+    <col min="12" max="12" width="2.7265625" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -62652,20 +62485,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2238422-2A43-47D2-83B8-E63DF0919ACF}">
   <dimension ref="C1:T156"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -66678,20 +66511,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:T157"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -70724,20 +70557,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="C1:T157"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="62.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="62.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>
@@ -74825,20 +74658,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:T157"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="1.7109375" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="2.28515625" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="15" max="17" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="1.7265625" customWidth="1"/>
+    <col min="3" max="3" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="2.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" customWidth="1"/>
+    <col min="15" max="17" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:19" ht="15.75" thickBot="1"/>
-    <row r="2" spans="3:19" ht="15.75" thickBot="1">
+    <row r="1" spans="3:19" ht="15" thickBot="1"/>
+    <row r="2" spans="3:19" ht="15" thickBot="1">
       <c r="C2" s="63" t="str">
         <f>"Financial Statement Model for "&amp;D5</f>
         <v>Financial Statement Model for Apple</v>

</xml_diff>